<commit_message>
Upgrade workbook tests for v0.44
- Fix errors and add new wrappers
- Add workbooks for new modules
  - fra
  - multicurve
  - varianceswaps
- Update defaultprobability workbook for trade_date argument
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/extras/example_interest_rate_derivatives.xlsx
+++ b/tests/workbooktests/workbooks/extras/example_interest_rate_derivatives.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\extras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E1ECC03-BFAD-403D-B7EE-D449B933C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2159AED3-B6B2-4DBE-81C4-5D98F357DCDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14655" yWindow="-20355" windowWidth="22170" windowHeight="15285" xr2:uid="{E29E0D93-B81D-4342-8E54-9A3C89952B2B}"/>
+    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{E29E0D93-B81D-4342-8E54-9A3C89952B2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="5" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C10" s="20" t="str" cm="1">
         <f t="array" ref="C10">_xll.qlVersion()</f>
-        <v>1.43</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.3">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="C11" s="20" t="str" cm="1">
         <f t="array" ref="C11">_xll.qlXlOilVersion()</f>
-        <v>0.43.0</v>
+        <v>0.44.0rc1</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.3">
@@ -2419,7 +2419,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G58" s="26" t="str" cm="1">
-        <f t="array" ref="G58">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F58,E58,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
+        <f t="array" ref="G58">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F58,E58,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,,,,,,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R58C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I58" s="27" cm="1">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="J58" s="28" cm="1">
         <f t="array" ref="J58">_xll.qlYieldTermStructureZeroRate($C$74,I58,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9056934878278965E-2</v>
+        <v>1.905693487827918E-2</v>
       </c>
       <c r="L58" s="28" cm="1">
         <f t="array" ref="L58">_xll.qlYieldTermStructureZeroRate($C$14,I58,"Act/365","Continuous","NoFrequency",TRUE)</f>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="M58" s="49">
         <f t="shared" ref="M58:M65" si="0">J58-L58</f>
-        <v>-3.6639466240353039E-4</v>
+        <v>-3.6639466240331528E-4</v>
       </c>
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.3">
@@ -2453,7 +2453,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G59" s="31" t="str" cm="1">
-        <f t="array" ref="G59">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F59,E59,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
+        <f t="array" ref="G59">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F59,E59,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,,,,,,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R59C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I59" s="32" cm="1">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="J59" s="33" cm="1">
         <f t="array" ref="J59">_xll.qlYieldTermStructureZeroRate($C$74,I59,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9341237502176117E-2</v>
+        <v>1.9341237502176225E-2</v>
       </c>
       <c r="L59" s="33" cm="1">
         <f t="array" ref="L59">_xll.qlYieldTermStructureZeroRate($C$14,I59,"Act/365","Continuous","NoFrequency",TRUE)</f>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="M59" s="50">
         <f t="shared" si="0"/>
-        <v>-3.6618246824472039E-4</v>
+        <v>-3.6618246824461284E-4</v>
       </c>
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.3">
@@ -2487,7 +2487,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G60" s="31" t="str" cm="1">
-        <f t="array" ref="G60">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F60,E60,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
+        <f t="array" ref="G60">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F60,E60,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,,,,,,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R60C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I60" s="32" cm="1">
@@ -2522,7 +2522,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G61" s="31" t="str" cm="1">
-        <f t="array" ref="G61">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F61,E61,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
+        <f t="array" ref="G61">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F61,E61,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,,,,,,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R61C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I61" s="32" cm="1">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="J61" s="33" cm="1">
         <f t="array" ref="J61">_xll.qlYieldTermStructureZeroRate($C$74,I61,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.0690783526765087E-2</v>
+        <v>2.0690783526765188E-2</v>
       </c>
       <c r="L61" s="33" cm="1">
         <f t="array" ref="L61">_xll.qlYieldTermStructureZeroRate($C$14,I61,"Act/365","Continuous","NoFrequency",TRUE)</f>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="M61" s="50">
         <f t="shared" si="0"/>
-        <v>-3.6583089206045777E-4</v>
+        <v>-3.6583089206035715E-4</v>
       </c>
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.3">
@@ -2557,7 +2557,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G62" s="31" t="str" cm="1">
-        <f t="array" ref="G62">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F62,E62,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
+        <f t="array" ref="G62">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F62,E62,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,,,,,,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R62C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I62" s="32" cm="1">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="J62" s="33" cm="1">
         <f t="array" ref="J62">_xll.qlYieldTermStructureZeroRate($C$74,I62,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.1438592526394247E-2</v>
+        <v>2.1438592526394289E-2</v>
       </c>
       <c r="L62" s="33" cm="1">
         <f t="array" ref="L62">_xll.qlYieldTermStructureZeroRate($C$14,I62,"Act/365","Continuous","NoFrequency",TRUE)</f>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="M62" s="50">
         <f t="shared" si="0"/>
-        <v>-3.657193791154166E-4</v>
+        <v>-3.6571937911537497E-4</v>
       </c>
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.3">
@@ -2592,7 +2592,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G63" s="31" t="str" cm="1">
-        <f t="array" ref="G63">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F63,E63,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
+        <f t="array" ref="G63">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F63,E63,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,,,,,,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R63C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I63" s="32" cm="1">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="J63" s="33" cm="1">
         <f t="array" ref="J63">_xll.qlYieldTermStructureZeroRate($C$74,I63,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.2939847920213422E-2</v>
+        <v>2.2939847920213502E-2</v>
       </c>
       <c r="L63" s="33" cm="1">
         <f t="array" ref="L63">_xll.qlYieldTermStructureZeroRate($C$14,I63,"Act/365","Continuous","NoFrequency",TRUE)</f>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="M63" s="50">
         <f t="shared" si="0"/>
-        <v>-3.6553547878125092E-4</v>
+        <v>-3.6553547878117112E-4</v>
       </c>
     </row>
     <row r="64" spans="2:13" x14ac:dyDescent="0.3">
@@ -2626,7 +2626,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G64" s="31" t="str" cm="1">
-        <f t="array" ref="G64">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F64,E64,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
+        <f t="array" ref="G64">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F64,E64,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,,,,,,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R64C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I64" s="32" cm="1">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="J64" s="33" cm="1">
         <f t="array" ref="J64">_xll.qlYieldTermStructureZeroRate($C$74,I64,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.5029132269805833E-2</v>
+        <v>2.502913226980585E-2</v>
       </c>
       <c r="L64" s="33" cm="1">
         <f t="array" ref="L64">_xll.qlYieldTermStructureZeroRate($C$14,I64,"Act/365","Continuous","NoFrequency",TRUE)</f>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="M64" s="50">
         <f t="shared" si="0"/>
-        <v>-3.6530716110095077E-4</v>
+        <v>-3.6530716110093342E-4</v>
       </c>
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.3">
@@ -2660,7 +2660,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G65" s="36" t="str" cm="1">
-        <f t="array" ref="G65">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F65,E65,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
+        <f t="array" ref="G65">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F65,E65,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,,,,,,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R65C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I65" s="37" cm="1">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="G80" s="49">
         <f>F80-M58</f>
-        <v>3.7880109931810083E-2</v>
+        <v>3.7880109931809874E-2</v>
       </c>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.3">
@@ -2806,8 +2806,8 @@
         <v>3.4626290911888569E-2</v>
       </c>
       <c r="G81" s="50">
-        <f>F81-M58</f>
-        <v>3.4992685574292096E-2</v>
+        <f t="shared" ref="G81:G88" si="2">F81-M58</f>
+        <v>3.4992685574291887E-2</v>
       </c>
     </row>
     <row r="82" spans="2:7" x14ac:dyDescent="0.3">
@@ -2827,8 +2827,8 @@
         <v>3.2751768392570955E-2</v>
       </c>
       <c r="G82" s="50">
-        <f>F82-M59</f>
-        <v>3.3117950860815676E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.3117950860815565E-2</v>
       </c>
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.3">
@@ -2841,7 +2841,7 @@
         <v>3.2377367024610644E-2</v>
       </c>
       <c r="G83" s="50">
-        <f>F83-M60</f>
+        <f t="shared" si="2"/>
         <v>3.2743326565338252E-2</v>
       </c>
     </row>
@@ -2855,8 +2855,8 @@
         <v>3.2661635352545959E-2</v>
       </c>
       <c r="G84" s="50">
-        <f>F84-M61</f>
-        <v>3.3027466244606417E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.3027466244606313E-2</v>
       </c>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.3">
@@ -2869,8 +2869,8 @@
         <v>3.3148897734764607E-2</v>
       </c>
       <c r="G85" s="50">
-        <f>F85-M62</f>
-        <v>3.3514617113880027E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.3514617113879985E-2</v>
       </c>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.3">
@@ -2883,8 +2883,8 @@
         <v>3.4367701312975452E-2</v>
       </c>
       <c r="G86" s="50">
-        <f>F86-M63</f>
-        <v>3.4733236791756703E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.4733236791756619E-2</v>
       </c>
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.3">
@@ -2897,8 +2897,8 @@
         <v>3.6219561600085722E-2</v>
       </c>
       <c r="G87" s="50">
-        <f>F87-M64</f>
-        <v>3.6584868761186676E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.6584868761186655E-2</v>
       </c>
     </row>
     <row r="88" spans="2:7" x14ac:dyDescent="0.3">
@@ -2911,7 +2911,7 @@
         <v>3.7390996111162984E-2</v>
       </c>
       <c r="G88" s="51">
-        <f>F88-M65</f>
+        <f t="shared" si="2"/>
         <v>3.7756178022948492E-2</v>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
         <v>77</v>
       </c>
       <c r="C16" s="36" t="str" cm="1">
-        <f t="array" ref="C16">_xll.xloRef(_xll.qlIborLeg(10000,C9,C11,"Act/360",,,,,,,,C12))</f>
+        <f t="array" ref="C16">_xll.xloRef(_xll.qlIborLeg(10000,C9,C11,"Act/360"))</f>
         <v>永[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3,A</v>
       </c>
       <c r="G16" s="2">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="C23" s="66" cm="1">
         <f t="array" ref="C23">_xll.qlInstrumentNPV(C18,_xll.qlInstrumentSetPricingEngine(C18,C21))</f>
-        <v>-457.45759571020835</v>
+        <v>-243.64750302948005</v>
       </c>
       <c r="G23" s="2">
         <v>46696</v>
@@ -7012,7 +7012,7 @@
       </c>
       <c r="X17" s="28" cm="1">
         <f t="array" ref="X17:X26">_xll.qlGsrVolatility(C31,C43)</f>
-        <v>7.2562982901529325E-3</v>
+        <v>7.2562982901533532E-3</v>
       </c>
     </row>
     <row r="18" spans="2:24" x14ac:dyDescent="0.3">
@@ -7094,7 +7094,7 @@
         <v>1</v>
       </c>
       <c r="X18" s="33">
-        <v>7.2854447762798731E-3</v>
+        <v>7.285444776279305E-3</v>
       </c>
     </row>
     <row r="19" spans="2:24" x14ac:dyDescent="0.3">
@@ -7176,7 +7176,7 @@
         <v>1</v>
       </c>
       <c r="X19" s="33">
-        <v>7.3317640293017773E-3</v>
+        <v>7.331764029302093E-3</v>
       </c>
     </row>
     <row r="20" spans="2:24" x14ac:dyDescent="0.3">
@@ -7251,7 +7251,7 @@
         <v>1</v>
       </c>
       <c r="X20" s="33">
-        <v>7.2499818707807877E-3</v>
+        <v>7.2499818707806273E-3</v>
       </c>
     </row>
     <row r="21" spans="2:24" x14ac:dyDescent="0.3">
@@ -7332,7 +7332,7 @@
         <v>1</v>
       </c>
       <c r="X21" s="33">
-        <v>7.0519393916380711E-3</v>
+        <v>7.0519393916377701E-3</v>
       </c>
     </row>
     <row r="22" spans="2:24" x14ac:dyDescent="0.3">
@@ -7413,7 +7413,7 @@
         <v>1</v>
       </c>
       <c r="X22" s="33">
-        <v>7.0789799045768848E-3</v>
+        <v>7.078979904577805E-3</v>
       </c>
     </row>
     <row r="23" spans="2:24" x14ac:dyDescent="0.3">
@@ -7488,7 +7488,7 @@
         <v>1</v>
       </c>
       <c r="X23" s="33">
-        <v>6.9660793842538805E-3</v>
+        <v>6.9660793842533028E-3</v>
       </c>
     </row>
     <row r="24" spans="2:24" x14ac:dyDescent="0.3">
@@ -7563,7 +7563,7 @@
         <v>1</v>
       </c>
       <c r="X24" s="33">
-        <v>7.8011054462023364E-3</v>
+        <v>7.8011054462026235E-3</v>
       </c>
     </row>
     <row r="25" spans="2:24" x14ac:dyDescent="0.3">
@@ -7638,7 +7638,7 @@
         <v>1</v>
       </c>
       <c r="X25" s="33">
-        <v>6.4311298987523163E-3</v>
+        <v>6.4311298987532678E-3</v>
       </c>
     </row>
     <row r="26" spans="2:24" x14ac:dyDescent="0.3">
@@ -7811,11 +7811,11 @@
       </c>
       <c r="C53" s="87" cm="1">
         <f t="array" ref="C53">_xll.qlInstrumentNPV(L17,_xll.qlInstrumentSetPricingEngine(L17,$C$32,$C$43))</f>
-        <v>480.19295857890654</v>
+        <v>480.19295857891234</v>
       </c>
       <c r="D53" s="87" cm="1">
         <f t="array" ref="D53">_xll.qlInstrumentNPV(L17,_xll.qlInstrumentSetPricingEngine(L17,$C$33,$C$43))</f>
-        <v>477.74924495888234</v>
+        <v>480.192958623089</v>
       </c>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.3">
@@ -7825,11 +7825,11 @@
       </c>
       <c r="C54" s="89" cm="1">
         <f t="array" ref="C54">_xll.qlInstrumentNPV(L18,_xll.qlInstrumentSetPricingEngine(L18,$C$32,$C$43))</f>
-        <v>514.75686806025317</v>
+        <v>514.75686806025544</v>
       </c>
       <c r="D54" s="89" cm="1">
         <f t="array" ref="D54">_xll.qlInstrumentNPV(L18,_xll.qlInstrumentSetPricingEngine(L18,$C$33,$C$43))</f>
-        <v>513.50611040521835</v>
+        <v>514.75686816147265</v>
       </c>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.3">
@@ -7839,11 +7839,11 @@
       </c>
       <c r="C55" s="89" cm="1">
         <f t="array" ref="C55">_xll.qlInstrumentNPV(L19,_xll.qlInstrumentSetPricingEngine(L19,$C$32,$C$43))</f>
-        <v>519.21992874969453</v>
+        <v>519.21992874970408</v>
       </c>
       <c r="D55" s="89" cm="1">
         <f t="array" ref="D55">_xll.qlInstrumentNPV(L19,_xll.qlInstrumentSetPricingEngine(L19,$C$33,$C$43))</f>
-        <v>517.23545516948286</v>
+        <v>519.21992893980871</v>
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
@@ -7853,11 +7853,11 @@
       </c>
       <c r="C56" s="89" cm="1">
         <f t="array" ref="C56">_xll.qlInstrumentNPV(L20,_xll.qlInstrumentSetPricingEngine(L20,$C$32,$C$43))</f>
-        <v>493.60804779991349</v>
+        <v>493.60804779989621</v>
       </c>
       <c r="D56" s="89" cm="1">
         <f t="array" ref="D56">_xll.qlInstrumentNPV(L20,_xll.qlInstrumentSetPricingEngine(L20,$C$33,$C$43))</f>
-        <v>491.03774318071919</v>
+        <v>493.60804829658883</v>
       </c>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.3">
@@ -7867,11 +7867,11 @@
       </c>
       <c r="C57" s="89" cm="1">
         <f t="array" ref="C57">_xll.qlInstrumentNPV(L21,_xll.qlInstrumentSetPricingEngine(L21,$C$32,$C$43))</f>
-        <v>445.12383139248038</v>
+        <v>445.12383139245065</v>
       </c>
       <c r="D57" s="89" cm="1">
         <f t="array" ref="D57">_xll.qlInstrumentNPV(L21,_xll.qlInstrumentSetPricingEngine(L21,$C$33,$C$43))</f>
-        <v>442.42184610809704</v>
+        <v>445.12383176478102</v>
       </c>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.3">
@@ -7881,11 +7881,11 @@
       </c>
       <c r="C58" s="89" cm="1">
         <f t="array" ref="C58">_xll.qlInstrumentNPV(L22,_xll.qlInstrumentSetPricingEngine(L22,$C$32,$C$43))</f>
-        <v>378.66930593822264</v>
+        <v>378.66930593828437</v>
       </c>
       <c r="D58" s="89" cm="1">
         <f t="array" ref="D58">_xll.qlInstrumentNPV(L22,_xll.qlInstrumentSetPricingEngine(L22,$C$33,$C$43))</f>
-        <v>376.09095103371908</v>
+        <v>378.6693062079907</v>
       </c>
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.3">
@@ -7895,11 +7895,11 @@
       </c>
       <c r="C59" s="89" cm="1">
         <f t="array" ref="C59">_xll.qlInstrumentNPV(L23,_xll.qlInstrumentSetPricingEngine(L23,$C$32,$C$43))</f>
-        <v>298.39373179886041</v>
+        <v>298.39373179893869</v>
       </c>
       <c r="D59" s="89" cm="1">
         <f t="array" ref="D59">_xll.qlInstrumentNPV(L23,_xll.qlInstrumentSetPricingEngine(L23,$C$33,$C$43))</f>
-        <v>296.23172499493859</v>
+        <v>298.39373204730759</v>
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
@@ -7909,11 +7909,11 @@
       </c>
       <c r="C60" s="89" cm="1">
         <f t="array" ref="C60">_xll.qlInstrumentNPV(L24,_xll.qlInstrumentSetPricingEngine(L24,$C$32,$C$43))</f>
-        <v>208.86665999869419</v>
+        <v>208.86665999882555</v>
       </c>
       <c r="D60" s="89" cm="1">
         <f t="array" ref="D60">_xll.qlInstrumentNPV(L24,_xll.qlInstrumentSetPricingEngine(L24,$C$33,$C$43))</f>
-        <v>207.31794600871279</v>
+        <v>208.86666035971777</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
@@ -7923,11 +7923,11 @@
       </c>
       <c r="C61" s="89" cm="1">
         <f t="array" ref="C61">_xll.qlInstrumentNPV(L25,_xll.qlInstrumentSetPricingEngine(L25,$C$32,$C$43))</f>
-        <v>107.37144562488741</v>
+        <v>107.37144562488729</v>
       </c>
       <c r="D61" s="89" cm="1">
         <f t="array" ref="D61">_xll.qlInstrumentNPV(L25,_xll.qlInstrumentSetPricingEngine(L25,$C$33,$C$43))</f>
-        <v>106.57878015619599</v>
+        <v>107.37144592013213</v>
       </c>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.3">
@@ -7937,7 +7937,7 @@
       <c r="C62" s="34"/>
       <c r="D62" s="91" cm="1">
         <f t="array" ref="D62">_xll.qlInstrumentNPV(C48,_xll.qlInstrumentSetPricingEngine(C48,$C$33,$C$43))</f>
-        <v>631.27448041042044</v>
+        <v>634.79544719393812</v>
       </c>
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.3">
@@ -7947,7 +7947,7 @@
       <c r="C64" s="120"/>
       <c r="D64" s="121">
         <f>D62-MAX(D53:D61)</f>
-        <v>114.03902524093758</v>
+        <v>115.57551825412941</v>
       </c>
     </row>
   </sheetData>

</xml_diff>